<commit_message>
Update for ICC estimation, new sheet to the Excel fila combining country and domain level info, new gamma column to show pop distribution by domain.
</commit_message>
<xml_diff>
--- a/tables/variables-2.xlsx
+++ b/tables/variables-2.xlsx
@@ -5322,7 +5322,7 @@
         <v>0.861</v>
       </c>
       <c r="R65" t="n">
-        <v>0.867</v>
+        <v>0.866</v>
       </c>
       <c r="S65" t="n">
         <v>0.994</v>
@@ -5337,7 +5337,7 @@
         <v>0.99</v>
       </c>
       <c r="W65" t="n">
-        <v>0.995</v>
+        <v>0.994</v>
       </c>
     </row>
     <row r="66">

</xml_diff>